<commit_message>
docs: synchronize note studio design memory
</commit_message>
<xml_diff>
--- a/docs/programs/NAS_NOTE_STUDIO_SPEC.xlsx
+++ b/docs/programs/NAS_NOTE_STUDIO_SPEC.xlsx
@@ -2,39 +2,39 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6eb9562bd73347cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Vision" sheetId="2" r:id="Rc330c3c8bff6484b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="3" r:id="Re3dbab34dbd845f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitors" sheetId="4" r:id="R07214adc71b04621"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open_Source" sheetId="5" r:id="Rb5e5b6e489a2495b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Index" sheetId="6" r:id="R9898689c65fb4fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Information_Architecture" sheetId="7" r:id="R37143fb679d34166"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_Layout" sheetId="8" r:id="Rc581f4ff979047a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User_Flows" sheetId="9" r:id="R99f2ec4db0b943a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note_Types" sheetId="10" r:id="Rb913225d6e714a37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Block_Catalog" sheetId="11" r:id="R0a7ef228309a4d44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slash_Commands" sheetId="12" r:id="R77baacb8b22d4f69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Menus" sheetId="13" r:id="R47e5083b9248485c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard_Shortcuts" sheetId="14" r:id="Rdbd2bfeb347d4ef0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Views" sheetId="15" r:id="R38047d44febd4700"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Text_Mode" sheetId="16" r:id="Ra0ecd9ce3c274194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python_Notebook" sheetId="17" r:id="R8d2ba8f1f2584e66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collaboration" sheetId="18" r:id="R857815610de946f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offline_Desktop" sheetId="19" r:id="R816e29109cb04a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Model" sheetId="20" r:id="R0368505a3bf7440b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage_Interop" sheetId="21" r:id="R632a10277d1b4934"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="22" r:id="R5cab643f232542d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Contracts" sheetId="23" r:id="Rfab52d5351404976"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State_Machines" sheetId="24" r:id="R58231673952f4755"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Error_Recovery" sheetId="25" r:id="R95645907a75f4bc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cross_App_Relations" sheetId="26" r:id="Rd7e9f1d3be03458d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="27" r:id="R4c138d69bb8d474a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accessibility" sheetId="28" r:id="Rf8d9dbaf56994bdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Matrix" sheetId="29" r:id="R88e9ae293c9e46ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="30" r:id="Rc76b38112fed49aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open_Questions" sheetId="31" r:id="R387c0f40ea554af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="32" r:id="Rfda4fa5dd3444472"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation_Status" sheetId="33" r:id="R797d2953039f4439"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R33e105af35254e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Vision" sheetId="2" r:id="Rbff19c2ac483427a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="3" r:id="Radf2fad0283842bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitors" sheetId="4" r:id="R1121be17aeb542c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open_Source" sheetId="5" r:id="Raac83768e7fe45a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Index" sheetId="6" r:id="Rc870cd1eed094d14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Information_Architecture" sheetId="7" r:id="R7a80a97d14ce471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_Layout" sheetId="8" r:id="R79405ef728dd4b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User_Flows" sheetId="9" r:id="R7923f8063aa34fa7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Note_Types" sheetId="10" r:id="R39a4b8b6a4fa4b41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Block_Catalog" sheetId="11" r:id="R3fabb14ac30c448c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slash_Commands" sheetId="12" r:id="R57abd8c952a447ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Menus" sheetId="13" r:id="Rd9a239a87d254b98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyboard_Shortcuts" sheetId="14" r:id="R654dcb37a5a64281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Views" sheetId="15" r:id="R84f7d5a8d3754a58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Text_Mode" sheetId="16" r:id="R8628dc79dc9e48bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python_Notebook" sheetId="17" r:id="Rf492ada1743d4f19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collaboration" sheetId="18" r:id="R757a3e35bb484ec6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offline_Desktop" sheetId="19" r:id="Rc8102fcef9604dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Model" sheetId="20" r:id="Rd562f07847ec42ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage_Interop" sheetId="21" r:id="Rbe8a0d902e864a3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="22" r:id="Ree6e6f88c1554c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Contracts" sheetId="23" r:id="Ra95ffcfad5914e1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State_Machines" sheetId="24" r:id="R8dd9a86f87cf4d32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Error_Recovery" sheetId="25" r:id="Rbac6869efdbb4422"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cross_App_Relations" sheetId="26" r:id="R968beef32bdf4912"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="27" r:id="R6b76cbf2ca884b6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accessibility" sheetId="28" r:id="R5cd7c64750e64886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Matrix" sheetId="29" r:id="Rbf78a13943e3411e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="30" r:id="R81c9f4429595416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open_Questions" sheetId="31" r:id="Rf5654a5927524968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="32" r:id="Rda03175fda5d4556"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation_Status" sheetId="33" r:id="R920fb7b5b5db4b92"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -928,7 +928,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d03bbbbf8ec4e6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12d4df722e2444b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1228,10 +1228,50 @@
         <x:v>M2</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="13" t="str">
+        <x:v>python-page</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="str">
+        <x:v>Python 실행 페이지</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>텍스트·제목·목록·파일·하위 페이지·Office 문서 reference와 실행 Python 셀을 섞는 rich page</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="str">
+        <x:v>Block canvas + cell editor + NAS kernel</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>MSP page/IPYNB/분리 PY+MD projection</x:v>
+      </x:c>
+      <x:c r="F15" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="str">
+        <x:v>notebook-root</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>노트북 작업공간</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>페이지 트리, 일반 파일, src/data/notebooks/references, 환경 선언을 담는 사용자 루트 폴더</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="str">
+        <x:v>Tree + file/page adapters</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>일반 폴더 bundle/manifest</x:v>
+      </x:c>
+      <x:c r="F16" s="13" t="str">
+        <x:v>M1 확장</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e2e1e9c7e9748bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdec4f685a2ed41a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1571,10 +1611,70 @@
         <x:v>M3</x:v>
       </x:c>
     </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="str">
+        <x:v>Structure</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="str">
+        <x:v>Office document reference</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="str">
+        <x:v>/document 또는 우클릭 삽입 &gt; 문서 만들기</x:v>
+      </x:c>
+      <x:c r="D17" s="13" t="str">
+        <x:v>DOCX/XLSX/PPTX/HWP/HWPX 생성, stable document ID, 현재 경로·저장 상태, 클릭 전면 열기</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>Markdown fallback link + manifest</x:v>
+      </x:c>
+      <x:c r="F17" s="13" t="str">
+        <x:v>M1 확장</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="13" t="str">
+        <x:v>Collaboration</x:v>
+      </x:c>
+      <x:c r="B18" s="13" t="str">
+        <x:v>Comment anchor</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="str">
+        <x:v>선택 후 댓글 또는 Ctrl+Shift+M</x:v>
+      </x:c>
+      <x:c r="D18" s="13" t="str">
+        <x:v>페이지·block·inline·code range thread, 답글, mention, resolve/reopen</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str">
+        <x:v>본문 export에서 기본 제외, 별도 comment archive 선택</x:v>
+      </x:c>
+      <x:c r="F18" s="13" t="str">
+        <x:v>M1.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="13" t="str">
+        <x:v>Code</x:v>
+      </x:c>
+      <x:c r="B19" s="13" t="str">
+        <x:v>Rich Python page blocks</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="str">
+        <x:v>/python-cell과 일반 block 혼합</x:v>
+      </x:c>
+      <x:c r="D19" s="13" t="str">
+        <x:v>실행기는 Python cell만 순서대로 실행하고 문서·링크·버튼 block은 실행하지 않음</x:v>
+      </x:c>
+      <x:c r="E19" s="13" t="str">
+        <x:v>IPYNB 또는 PY+MD+manifest</x:v>
+      </x:c>
+      <x:c r="F19" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46460ecb1a4e4a9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb31bd394658453b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1894,10 +1994,70 @@
         <x:v>M3</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="str">
+        <x:v>파일·문서</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>/document</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>문서 만들기</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="str">
+        <x:v>현재 caret/block 또는 선택 폴더</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>DOCX/XLSX/PPTX/HWP/HWPX 선택 후 draft 생성</x:v>
+      </x:c>
+      <x:c r="F16" s="13" t="str">
+        <x:v>M1 확장</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="str">
+        <x:v>파일·문서</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="str">
+        <x:v>/link-document</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="str">
+        <x:v>기존 NAS 문서 연결</x:v>
+      </x:c>
+      <x:c r="D17" s="13" t="str">
+        <x:v>note edit + file read 권한</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>stable document reference block 삽입</x:v>
+      </x:c>
+      <x:c r="F17" s="13" t="str">
+        <x:v>M1 확장</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="13" t="str">
+        <x:v>협업</x:v>
+      </x:c>
+      <x:c r="B18" s="13" t="str">
+        <x:v>/comment</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="str">
+        <x:v>선택 영역에 댓글</x:v>
+      </x:c>
+      <x:c r="D18" s="13" t="str">
+        <x:v>comment 권한과 selection</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str">
+        <x:v>anchor thread 열기</x:v>
+      </x:c>
+      <x:c r="F18" s="13" t="str">
+        <x:v>M1.5</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f833838b4734d98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb4cf5bb05014f0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2239,10 +2399,78 @@
         <x:v>삭제된 파일은 broken reference와 복구 경로</x:v>
       </x:c>
     </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="13" t="str">
+        <x:v>노트북 폴더/파일 영역</x:v>
+      </x:c>
+      <x:c r="B20" s="13" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C20" s="13" t="str">
+        <x:v>새 페이지 / 새 폴더 / 문서 만들기</x:v>
+      </x:c>
+      <x:c r="D20" s="13" t="str">
+        <x:v>생성 권한</x:v>
+      </x:c>
+      <x:c r="E20" s="13" t="str">
+        <x:v>우클릭한 invocation directory를 draft 기본 저장 위치로 기억</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="13" t="str">
+        <x:v>블록 핸들/본문 caret</x:v>
+      </x:c>
+      <x:c r="B21" s="13" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="str">
+        <x:v>하위 페이지 / Office 문서 / 기존 NAS 문서 연결</x:v>
+      </x:c>
+      <x:c r="D21" s="13" t="str">
+        <x:v>note edit + target create/read 권한</x:v>
+      </x:c>
+      <x:c r="E21" s="13" t="str">
+        <x:v>현재 위치에 page 또는 document reference block 삽입</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="13" t="str">
+        <x:v>문서 reference</x:v>
+      </x:c>
+      <x:c r="B22" s="13" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="str">
+        <x:v>열기 / NAS에서 보기 / 위치 복사 / 다시 연결</x:v>
+      </x:c>
+      <x:c r="D22" s="13" t="str">
+        <x:v>대상 read 권한</x:v>
+      </x:c>
+      <x:c r="E22" s="13" t="str">
+        <x:v>지원 편집기를 전면 열고 stable ID를 서버에서 재해석</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="13" t="str">
+        <x:v>문서 reference</x:v>
+      </x:c>
+      <x:c r="B23" s="13" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C23" s="13" t="str">
+        <x:v>링크 제거 / 링크와 파일 함께 삭제</x:v>
+      </x:c>
+      <x:c r="D23" s="13" t="str">
+        <x:v>note edit; 실제 삭제는 file delete 권한</x:v>
+      </x:c>
+      <x:c r="E23" s="13" t="str">
+        <x:v>기본은 링크만 제거. 함께 삭제는 확인 후 휴지통</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab5ccac86a3848d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf599bc839e914f09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2740,7 +2968,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4842afea2bc43f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1c0ea63ec7f49e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3000,7 +3228,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f2d23d8dd6a4631"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60e20feff95e4feb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3192,7 +3420,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b74bee02a7f4399"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c29b0107ef041e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3449,10 +3677,78 @@
         <x:v>M2</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="13" t="str">
+        <x:v>혼합 페이지</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="str">
+        <x:v>일반 block + Python cell</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>페이지 링크·텍스트·이미지·Office reference와 code cell을 한 페이지에 배치하고 실행기는 code cell만 처리.</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="str">
+        <x:v>숨겨진 실행 상태와 block action이 코드로 섞이지 않음.</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="str">
+        <x:v>원격 실행</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>NAS workspace 실행</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>NAS 경로는 그대로 유지하고 PC는 편집·요청·stdout/stderr/rich output stream만 담당.</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="str">
+        <x:v>임의 로컬 앱 실행을 원격으로 가장하지 않고 공식 VS Code/Driver/Studio 관문만 지원.</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="str">
+        <x:v>자원 감지</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="str">
+        <x:v>동적 admission</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="str">
+        <x:v>매 배정 시 MemAvailable, CPU load, swap pressure, disk reserve, 온도, active/reserved 작업을 재측정.</x:v>
+      </x:c>
+      <x:c r="D17" s="13" t="str">
+        <x:v>현재 초기 전역 1·계정당 1. 증설은 OS 인식 후 계산하되 GPU capability는 MASTER 승인 전 차단.</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="13" t="str">
+        <x:v>로컬 투영</x:v>
+      </x:c>
+      <x:c r="B18" s="13" t="str">
+        <x:v>PY+MD+assets+manifest</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="str">
+        <x:v>stable block/cell marker, revision/hash/base snapshot으로 round-trip.</x:v>
+      </x:c>
+      <x:c r="D18" s="13" t="str">
+        <x:v>동시 수정은 자동 덮어쓰기 금지. rich-only block은 manifest 보존.</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0e1f34abeea4106"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1dca47cee9a4be0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3641,10 +3937,78 @@
         <x:v>unknown nodes round-trip 보존</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="13" t="str">
+        <x:v>댓글 범위</x:v>
+      </x:c>
+      <x:c r="B11" s="13" t="str">
+        <x:v>page discussion, block, inline text, Python cell/code range</x:v>
+      </x:c>
+      <x:c r="C11" s="13" t="str">
+        <x:v>NoteComment thread와 stable block/cell ID, 선택 anchor/context를 저장한다.</x:v>
+      </x:c>
+      <x:c r="D11" s="13" t="str">
+        <x:v>다른 계정·권한 회수 시 본문이나 댓글 preview를 노출하지 않는다.</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="str">
+        <x:v>M1.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="13" t="str">
+        <x:v>댓글 수명</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="str">
+        <x:v>답글·mention·알림·resolve/reopen·수정·삭제</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="str">
+        <x:v>작성자·시간·권한·감사를 보존하고 해결된 thread도 조회 가능하게 한다.</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="str">
+        <x:v>삭제 사용자 표시와 알림 중복 정책을 고정한다.</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="str">
+        <x:v>M1.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="13" t="str">
+        <x:v>anchor 복구</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>본문 또는 코드 변경 뒤 위치 추적</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>block ID와 앞뒤 문맥을 사용하고 확신할 수 없으면 위치 변경됨으로 표시한다.</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="str">
+        <x:v>비슷한 문장이 있어도 추측 재부착하지 않는다.</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>M1.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="13" t="str">
+        <x:v>실제 소스 주석</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="str">
+        <x:v>.py # 등 언어 문법</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="str">
+        <x:v>review thread와 분리해 로컬 파일 round-trip에 포함한다.</x:v>
+      </x:c>
+      <x:c r="D14" s="13" t="str">
+        <x:v>검토 댓글을 source text로 자동 삽입하지 않는다.</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5493f4fe73194ada"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra68c384b88a64abf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3836,7 +4200,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e59bcd9e60b43dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf067d158fbca4abd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3969,7 +4333,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85281a390ece445a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a117e9de74040dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4243,10 +4607,112 @@
         <x:v>높음</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="str">
+        <x:v>NotebookWorkspace</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>id, ownerUid, title, rootDirectoryId, schemaVersion, executionPolicy, timestamps</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>사용자 personal root 안의 stable directory identity와 연결</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="str">
+        <x:v>owner+rootDirectoryId</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>높음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="str">
+        <x:v>PageProjection</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="str">
+        <x:v>pageId, clientId, serverRevision, baseHash, pyPath, mdPath, manifestPath, status</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="str">
+        <x:v>서버 rich page가 기준이며 로컬 두 파일을 독립 원본으로 취급하지 않음</x:v>
+      </x:c>
+      <x:c r="D17" s="13" t="str">
+        <x:v>page+client+revision</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>높음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="13" t="str">
+        <x:v>DocumentIdentity</x:v>
+      </x:c>
+      <x:c r="B18" s="13" t="str">
+        <x:v>documentId, ownerUid, fileId, currentPath, revision, state</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="str">
+        <x:v>이동·이름 변경 후에도 같은 실제 파일을 가리킴</x:v>
+      </x:c>
+      <x:c r="D18" s="13" t="str">
+        <x:v>fileId/path 역색인</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str">
+        <x:v>높음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="13" t="str">
+        <x:v>DocumentReferenceBlock</x:v>
+      </x:c>
+      <x:c r="B19" s="13" t="str">
+        <x:v>blockId, noteId, documentId, displayName, lastKnownPath</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="str">
+        <x:v>대상 권한을 상속하거나 파일을 복제하지 않음</x:v>
+      </x:c>
+      <x:c r="D19" s="13" t="str">
+        <x:v>document backlink</x:v>
+      </x:c>
+      <x:c r="E19" s="13" t="str">
+        <x:v>높음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="13" t="str">
+        <x:v>CommentAnchor</x:v>
+      </x:c>
+      <x:c r="B20" s="13" t="str">
+        <x:v>threadId, blockId, cellId, from/to, quote, prefix, suffix, anchorState</x:v>
+      </x:c>
+      <x:c r="C20" s="13" t="str">
+        <x:v>불확실한 재부착 금지</x:v>
+      </x:c>
+      <x:c r="D20" s="13" t="str">
+        <x:v>thread+block/cell</x:v>
+      </x:c>
+      <x:c r="E20" s="13" t="str">
+        <x:v>높음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="13" t="str">
+        <x:v>ExecutionCapability</x:v>
+      </x:c>
+      <x:c r="B21" s="13" t="str">
+        <x:v>subjectId, capability, grantedByMaster, limits, expiresAt, revokedAt</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="str">
+        <x:v>GPU/CUDA/high-load 권한은 MASTER만 부여·회수</x:v>
+      </x:c>
+      <x:c r="D21" s="13" t="str">
+        <x:v>subject+capability</x:v>
+      </x:c>
+      <x:c r="E21" s="13" t="str">
+        <x:v>매우 높음</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb972bc0a30d349e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R934c0cfb873142b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4418,10 +4884,78 @@
         <x:v>STORAGE-CAPACITY-ALLOCATION</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="13" t="str">
+        <x:v>노트북 물리 루트</x:v>
+      </x:c>
+      <x:c r="B10" s="13" t="str">
+        <x:v>NOTE MANAGER/&lt;노트북 이름&gt;</x:v>
+      </x:c>
+      <x:c r="C10" s="13" t="str">
+        <x:v>페이지 marker가 있는 폴더와 일반 src/data/reference/env 파일을 함께 허용</x:v>
+      </x:c>
+      <x:c r="D10" s="13" t="str">
+        <x:v>노트북 밖 상대경로 이탈은 명시 연결 없이는 금지</x:v>
+      </x:c>
+      <x:c r="E10" s="13" t="str">
+        <x:v>M1 확장</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="13" t="str">
+        <x:v>Python 페이지 로컬 투영</x:v>
+      </x:c>
+      <x:c r="B11" s="13" t="str">
+        <x:v>&lt;페이지&gt;/&lt;페이지&gt;.py + .md + assets + .msp-page.json</x:v>
+      </x:c>
+      <x:c r="C11" s="13" t="str">
+        <x:v>PY에는 코드만, MD에는 표준 문서 block, 고급 block은 manifest</x:v>
+      </x:c>
+      <x:c r="D11" s="13" t="str">
+        <x:v>atomic write, hash, revision, base snapshot, conflict copy</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="13" t="str">
+        <x:v>환경 파일</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="str">
+        <x:v>.env.example 동기화, 실제 secret은 장치/서버 비밀 저장소</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="str">
+        <x:v>실행 때 환경변수로 주입하고 공유·Git·일반 동기화에서 제외</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="str">
+        <x:v>secret 포함 .env 자동 공유 금지</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="13" t="str">
+        <x:v>Office 문서 연결</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>호출 폴더 또는 사용자가 고른 계정 내 NAS 경로</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>실제 파일 하나와 stable document reference 사용</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="str">
+        <x:v>복제 금지, 이동·이름 변경 registry 갱신</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>M1 확장</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a43bc93831467d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42a7fa329dc54920"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4661,10 +5195,78 @@
         <x:v>P0</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="13" t="str">
+        <x:v>SEC-13</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="str">
+        <x:v>동적 실행 자원 고갈과 서비스 starvation</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="str">
+        <x:v>실제 cgroup/OS 지표 기반 예약 admission, 공정 대기열, 일반 서비스 reserve, timeout/OOM/출력 제한.</x:v>
+      </x:c>
+      <x:c r="D14" s="13" t="str">
+        <x:v>동시 사용자, swap 압박, disk full, 온도, worker crash 부하 테스트</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="13" t="str">
+        <x:v>SEC-14</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="str">
+        <x:v>GPU/CUDA·고부하 capability 오남용</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>기본 차단. MANAGER도 부여 불가, MASTER만 self-test·limit·만료를 포함해 계정별 허용.</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="str">
+        <x:v>권한 상승·만료·회수·감사 회귀</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="str">
+        <x:v>SEC-15</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>local projection이 서버/다른 변경을 덮어씀</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>base revision/hash 3-way merge, 원자 교체, 충돌 복사본, rich-only block 보존.</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="str">
+        <x:v>동시 NAS/PC 편집과 중단·재시작</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="str">
+        <x:v>SEC-16</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="str">
+        <x:v>Office draft가 다른 경로나 계정에 저장됨</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="str">
+        <x:v>invocation directory stable ID, first-save realpath/symlink/quota 재검증, 실패 시 위치 재선택.</x:v>
+      </x:c>
+      <x:c r="D17" s="13" t="str">
+        <x:v>폴더 이동·삭제·권한 회수·이름 충돌</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re80d3ed524f74eb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b80ddd6b52e4bb6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5023,10 +5625,112 @@
         <x:v>file read + note edit + quota</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="13" t="str">
+        <x:v>Notebook</x:v>
+      </x:c>
+      <x:c r="B21" s="13" t="str">
+        <x:v>POST /api/notebooks/:id/projections</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="str">
+        <x:v>clientId, serverRevision, formats, idempotencyKey</x:v>
+      </x:c>
+      <x:c r="D21" s="13" t="str">
+        <x:v>projection descriptor/job</x:v>
+      </x:c>
+      <x:c r="E21" s="13" t="str">
+        <x:v>read/edit 권한, revision precondition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="13" t="str">
+        <x:v>Notebook</x:v>
+      </x:c>
+      <x:c r="B22" s="13" t="str">
+        <x:v>POST /api/notebooks/:id/execution-admission</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="str">
+        <x:v>environment, requestedResources, capability</x:v>
+      </x:c>
+      <x:c r="D22" s="13" t="str">
+        <x:v>queued/reserved/denied와 이유</x:v>
+      </x:c>
+      <x:c r="E22" s="13" t="str">
+        <x:v>execute 권한, MASTER capability, request dedupe</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="13" t="str">
+        <x:v>Documents</x:v>
+      </x:c>
+      <x:c r="B23" s="13" t="str">
+        <x:v>POST /api/notes/:id/documents</x:v>
+      </x:c>
+      <x:c r="C23" s="13" t="str">
+        <x:v>format, invocationDirectoryId, caret/block anchor, draftId, idempotencyKey</x:v>
+      </x:c>
+      <x:c r="D23" s="13" t="str">
+        <x:v>draft/document reference descriptor</x:v>
+      </x:c>
+      <x:c r="E23" s="13" t="str">
+        <x:v>note edit + directory create + quota, 원자 생성/연결</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="13" t="str">
+        <x:v>Documents</x:v>
+      </x:c>
+      <x:c r="B24" s="13" t="str">
+        <x:v>POST /api/note-document-drafts/:id/publish</x:v>
+      </x:c>
+      <x:c r="C24" s="13" t="str">
+        <x:v>name, targetDirectoryId, expectedPageRevision</x:v>
+      </x:c>
+      <x:c r="D24" s="13" t="str">
+        <x:v>documentId, currentPath, reference block</x:v>
+      </x:c>
+      <x:c r="E24" s="13" t="str">
+        <x:v>realpath/quota/extension, 반복 publish 안전</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="13" t="str">
+        <x:v>Documents</x:v>
+      </x:c>
+      <x:c r="B25" s="13" t="str">
+        <x:v>GET /api/documents/:documentId/resolve</x:v>
+      </x:c>
+      <x:c r="C25" s="13" t="str">
+        <x:v>knownRevision</x:v>
+      </x:c>
+      <x:c r="D25" s="13" t="str">
+        <x:v>현재 path/state/editor kind</x:v>
+      </x:c>
+      <x:c r="E25" s="13" t="str">
+        <x:v>document read 권한, 경로 정보 최소화</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="13" t="str">
+        <x:v>Comments</x:v>
+      </x:c>
+      <x:c r="B26" s="13" t="str">
+        <x:v>PATCH /api/note-comments/:threadId</x:v>
+      </x:c>
+      <x:c r="C26" s="13" t="str">
+        <x:v>body/resolve/reopen/anchor repair</x:v>
+      </x:c>
+      <x:c r="D26" s="13" t="str">
+        <x:v>thread revision</x:v>
+      </x:c>
+      <x:c r="E26" s="13" t="str">
+        <x:v>author/comment 권한, If-Match</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ceb9b1bdaca47aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fb3a66fdd5541f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5337,7 +6041,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R151174993b6c49a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcddab77635e8401b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5560,10 +6264,95 @@
         <x:v>웹/WS/worker health</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="13" t="str">
+        <x:v>투영 중 NAS·PC 동시 수정</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>base snapshot 기준 코드·문서별 3-way diff</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>내 사본/서버 사본/수동 병합</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="str">
+        <x:v>양쪽과 rich-only manifest 보존</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>새 revision으로 명시 확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="13" t="str">
+        <x:v>Office 첫 저장 전 호출 폴더 이동·삭제</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="str">
+        <x:v>stable directory ID 재해석</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="str">
+        <x:v>새 NAS 위치 선택/초안 계속/취소</x:v>
+      </x:c>
+      <x:c r="D14" s="13" t="str">
+        <x:v>draft와 노트 본문 보존</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>원자 publish와 reference 생성</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="13" t="str">
+        <x:v>Office 파일 이동·이름 변경</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="str">
+        <x:v>document registry currentPath 갱신</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>NAS에서 보기/다시 연결</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="str">
+        <x:v>reference block과 backlink 유지</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>documentId resolve 성공</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="str">
+        <x:v>실행 admission 자원 부족</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>공정 queue와 지수 backoff 재평가</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>대기 취소/낮은 한도로 재요청</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="str">
+        <x:v>코드·문서·요청 metadata 보존</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>예약 후 시작 또는 명시 취소</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="str">
+        <x:v>장치 업그레이드·제거</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="str">
+        <x:v>metrics 즉시 갱신, 매 admission 실제 capacity 재계산</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="str">
+        <x:v>MASTER capability self-test/활성화</x:v>
+      </x:c>
+      <x:c r="D17" s="13" t="str">
+        <x:v>고부하 권한은 자동 확대하지 않음</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>OS 인식+검증 뒤 새 한도 적용</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R739e7f1623a3418d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f36de33024a4c40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5820,10 +6609,78 @@
         <x:v>채팅 지연이 편집 socket에 영향</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="13" t="str">
+        <x:v>DOCUMENT-WORKSPACE</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="str">
+        <x:v>reuses</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>빈 DOCX/XLSX/PPTX/HWP/HWPX 생성, quota, 원자 저장, OnlyOffice/RHWP 전면 열기</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="str">
+        <x:v>draft context와 note reference transaction, stable document ID</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>별도 생성 로직 분기로 형식·저장 오류 재발</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="str">
+        <x:v>DOCUMENT-STUDIO</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>integrates</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>노트/페이지/선택 내용의 변환·내보내기 job과 결과 열기</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="str">
+        <x:v>원본 block과 결과 file reference 관계</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>문서 변환과 문서 편집 앱 명칭 혼동</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="str">
+        <x:v>PC-LINK/DRIVE</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="str">
+        <x:v>projects</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="str">
+        <x:v>노트북 폴더 placeholder/hydration, local PY+MD projection, 변경 watcher</x:v>
+      </x:c>
+      <x:c r="D17" s="13" t="str">
+        <x:v>stable cell marker와 3-way merge, machine-local env 제외</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>생성 파일이 사용자 편집을 덮어씀</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="13" t="str">
+        <x:v>ADMIN-SERVER-MONITORING</x:v>
+      </x:c>
+      <x:c r="B18" s="13" t="str">
+        <x:v>feeds</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="str">
+        <x:v>CPU/RAM/swap/disk/temperature/장치 지표</x:v>
+      </x:c>
+      <x:c r="D18" s="13" t="str">
+        <x:v>실행 admission용 예약·압력·capability 상태</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str">
+        <x:v>표시 지표와 실제 scheduler 판단 불일치</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R824b3d2194894eca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9488069b7054ed4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6012,10 +6869,61 @@
         <x:v>Tauri/Electron 비교</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="13" t="str">
+        <x:v>PERF-10</x:v>
+      </x:c>
+      <x:c r="B11" s="13" t="str">
+        <x:v>동적 Python scheduler</x:v>
+      </x:c>
+      <x:c r="C11" s="13" t="str">
+        <x:v>현재 장비는 global active 1, user active 1부터 시작</x:v>
+      </x:c>
+      <x:c r="D11" s="13" t="str">
+        <x:v>여러 계정 queue + MemAvailable 3GiB대 + swap pressure</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="str">
+        <x:v>자원 예약, fair queue, 일반 서비스 reserve, 측정 후 경량 2개</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="13" t="str">
+        <x:v>PERF-11</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="str">
+        <x:v>장치 재감지</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="str">
+        <x:v>UI 5초 갱신, admission마다 실제 capacity 재계산</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="str">
+        <x:v>RAM/디스크 변화와 GPU 추가 mock/실장비</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="str">
+        <x:v>감소 즉시 보수화, GPU는 MASTER self-test 전 비활성</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="13" t="str">
+        <x:v>PERF-12</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>페이지 로컬 투영</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>변경된 block/cell만 재생성하고 5,000 block에서도 UI/동기화 정지 없음</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="str">
+        <x:v>NAS/PC 동시 편집, 대형 MD·PY·assets</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>incremental projection, hash cache, background merge</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fd4e69cfdba47d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb04ff36ac1a4f0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6176,7 +7084,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dc33a4070d64f13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R800dea6f13634c7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6576,10 +7484,130 @@
         <x:v>M3</x:v>
       </x:c>
     </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="13" t="str">
+        <x:v>T-019</x:v>
+      </x:c>
+      <x:c r="B20" s="13" t="str">
+        <x:v>혼합 Python 페이지</x:v>
+      </x:c>
+      <x:c r="C20" s="13" t="str">
+        <x:v>텍스트·링크·Office block 사이 code cell 실행/all/restart</x:v>
+      </x:c>
+      <x:c r="D20" s="13" t="str">
+        <x:v>code cell만 정확한 순서로 실행하고 문서 block은 실행되지 않음</x:v>
+      </x:c>
+      <x:c r="E20" s="13" t="str">
+        <x:v>integration+E2E</x:v>
+      </x:c>
+      <x:c r="F20" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="13" t="str">
+        <x:v>T-020</x:v>
+      </x:c>
+      <x:c r="B21" s="13" t="str">
+        <x:v>로컬 투영</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="str">
+        <x:v>서버 page와 PC의 .py/.md를 동시에 수정 후 sync</x:v>
+      </x:c>
+      <x:c r="D21" s="13" t="str">
+        <x:v>사용자 변경을 덮어쓰지 않고 block별 diff/충돌 복사본, rich metadata 보존</x:v>
+      </x:c>
+      <x:c r="E21" s="13" t="str">
+        <x:v>round-trip+E2E</x:v>
+      </x:c>
+      <x:c r="F21" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="13" t="str">
+        <x:v>T-021</x:v>
+      </x:c>
+      <x:c r="B22" s="13" t="str">
+        <x:v>댓글</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="str">
+        <x:v>inline/code range 댓글 뒤 본문 삽입·삭제·이동·resolve/reopen</x:v>
+      </x:c>
+      <x:c r="D22" s="13" t="str">
+        <x:v>anchor 복구 또는 위치 변경됨, 잘못된 재부착 없음</x:v>
+      </x:c>
+      <x:c r="E22" s="13" t="str">
+        <x:v>unit+E2E</x:v>
+      </x:c>
+      <x:c r="F22" s="13" t="str">
+        <x:v>M1.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="13" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="B23" s="13" t="str">
+        <x:v>Office 생성</x:v>
+      </x:c>
+      <x:c r="C23" s="13" t="str">
+        <x:v>본문 caret·폴더 우클릭에서 5개 형식 생성, 다른 위치 첫 저장</x:v>
+      </x:c>
+      <x:c r="D23" s="13" t="str">
+        <x:v>호출 위치 기본값, 실제 파일 1개, reference block, 편집기 전면 열기</x:v>
+      </x:c>
+      <x:c r="E23" s="13" t="str">
+        <x:v>integration+E2E</x:v>
+      </x:c>
+      <x:c r="F23" s="13" t="str">
+        <x:v>M1 확장</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="13" t="str">
+        <x:v>T-023</x:v>
+      </x:c>
+      <x:c r="B24" s="13" t="str">
+        <x:v>Office 저장 경계</x:v>
+      </x:c>
+      <x:c r="C24" s="13" t="str">
+        <x:v>호출 폴더 이동·삭제·권한 회수·quota full·이름 충돌</x:v>
+      </x:c>
+      <x:c r="D24" s="13" t="str">
+        <x:v>임의 fallback/덮어쓰기 없음, draft 보존, 위치 재선택·복구 가능</x:v>
+      </x:c>
+      <x:c r="E24" s="13" t="str">
+        <x:v>security+E2E</x:v>
+      </x:c>
+      <x:c r="F24" s="13" t="str">
+        <x:v>M1 확장</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="13" t="str">
+        <x:v>T-024</x:v>
+      </x:c>
+      <x:c r="B25" s="13" t="str">
+        <x:v>동적 자원</x:v>
+      </x:c>
+      <x:c r="C25" s="13" t="str">
+        <x:v>동시 Python, swap pressure, OOM, 장치 용량 증감</x:v>
+      </x:c>
+      <x:c r="D25" s="13" t="str">
+        <x:v>일반 서비스 정상, 작업 queue/kill/retry, 새 OS capacity 반영, GPU 권한 자동 개방 없음</x:v>
+      </x:c>
+      <x:c r="E25" s="13" t="str">
+        <x:v>security+load</x:v>
+      </x:c>
+      <x:c r="F25" s="13" t="str">
+        <x:v>M2</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f6784964ff343df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3db7627c174c40f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6785,10 +7813,146 @@
         <x:v>PWA 오프라인 프로토타입 및 파일시스템·딥링크·업데이트 요구 확정 후</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="13" t="str">
+        <x:v>DEC-011</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="str">
+        <x:v>채택</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="str">
+        <x:v>노트북은 사용자 계정 루트의 휴대 가능한 작업공간이며 모든 페이지 유형이 하위 페이지와 일반 파일을 함께 가질 수 있다.</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="str">
+        <x:v>Notion식 계층과 Python·Markdown·환경·참고 파일을 한 프로젝트 경계에서 다루기 위해서다.</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="str">
+        <x:v>파일 관리자와 노트 트리의 물리·논리 경계 spike에서 충돌할 때</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="13" t="str">
+        <x:v>DEC-012</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>채택</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>Python 실행 페이지는 문서 블록과 실행 코드 셀을 섞되 raw .py 파일은 순수 소스로 유지한다.</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="str">
+        <x:v>텍스트·링크·Office 문서 블록이 코드 실행을 오염시키지 않고 외부 Python 도구 호환성을 지킨다.</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>Jupyter round-trip에서 block metadata를 보존할 수 없을 때</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="13" t="str">
+        <x:v>DEC-013</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="str">
+        <x:v>채택</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="str">
+        <x:v>NAS의 rich block 페이지를 기준 원본으로 하고 로컬에는 .py·.md·assets·숨김 manifest 작업 폴더를 투영한다.</x:v>
+      </x:c>
+      <x:c r="D14" s="13" t="str">
+        <x:v>NAS에서는 한 페이지 UX를 유지하면서 로컬 VS Code·터미널·Markdown 앱에서 실제 파일로 작업한다.</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>양방향 병합이 안정적으로 구현되지 못할 때 읽기 전용 export로 축소</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="13" t="str">
+        <x:v>DEC-014</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="str">
+        <x:v>채택</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>표준 Markdown 기능은 양방향 보존하고 글꼴·버튼·database·실행 output 등 고급 블록은 manifest와 rich schema에 보존한다.</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="str">
+        <x:v>MDX/raw HTML에 임의 기능을 넣으면 외부 편집기 호환성과 XSS 경계가 깨진다.</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>안전하고 공개된 확장 문법을 채택할 때</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="13" t="str">
+        <x:v>DEC-015</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="str">
+        <x:v>채택</x:v>
+      </x:c>
+      <x:c r="C16" s="13" t="str">
+        <x:v>Python 원격 실행은 실제 OS/cgroup 자원 기반 admission queue와 격리 worker를 통과해야 한다.</x:v>
+      </x:c>
+      <x:c r="D16" s="13" t="str">
+        <x:v>저사양 NAS에서 동시 실행이 일반 파일·노트 서비스를 중단시키지 않아야 한다.</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>예외 없음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="13" t="str">
+        <x:v>DEC-016</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="str">
+        <x:v>채택</x:v>
+      </x:c>
+      <x:c r="C17" s="13" t="str">
+        <x:v>문서·블록·선택 텍스트·코드 줄 검토 댓글과 실제 소스 주석을 서로 다른 모델로 저장한다.</x:v>
+      </x:c>
+      <x:c r="D17" s="13" t="str">
+        <x:v>검토 대화가 .py/.md 본문을 바꾸지 않고 편집 후에도 안전하게 anchor를 추적해야 한다.</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>예외 없음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="13" t="str">
+        <x:v>DEC-017</x:v>
+      </x:c>
+      <x:c r="B18" s="13" t="str">
+        <x:v>채택</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="str">
+        <x:v>노트 본문과 트리의 문서 만들기는 기존 문서 스튜디오 생성·편집 서비스를 재사용한다.</x:v>
+      </x:c>
+      <x:c r="D18" s="13" t="str">
+        <x:v>별도 빈 Office 파일 생성기를 만들지 않고 계정 경계·quota·원자 저장·OnlyOffice/RHWP 검증을 공유한다.</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str">
+        <x:v>문서 스튜디오 API 계약이 교체될 때</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="13" t="str">
+        <x:v>DEC-018</x:v>
+      </x:c>
+      <x:c r="B19" s="13" t="str">
+        <x:v>채택</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="str">
+        <x:v>Office 문서 최초 저장 기본 위치는 명령이 발생한 노트북 내부 폴더이며 다른 NAS 위치 저장 후에도 stable document ID 링크를 유지한다.</x:v>
+      </x:c>
+      <x:c r="D19" s="13" t="str">
+        <x:v>Notion 하위 페이지 링크와 같은 본문 UX를 실제 NAS 파일에 적용하고 이동·이름 변경으로 링크가 깨지지 않게 한다.</x:v>
+      </x:c>
+      <x:c r="E19" s="13" t="str">
+        <x:v>stable file/document identity 저장소 설계 변경 시</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6adeabb1b1f4aa3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3c863aa22b740fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6929,7 +8093,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b8909fa322f4025"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R304c5770598843e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7138,7 +8302,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28c11dbc8cc54e77"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d1a53911fd54c43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7238,10 +8402,30 @@
         <x:v>Codex</x:v>
       </x:c>
     </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="13" t="str">
+        <x:v>2026-09-06</x:v>
+      </x:c>
+      <x:c r="B5" s="13" t="str">
+        <x:v>0.4-design-memory-sync</x:v>
+      </x:c>
+      <x:c r="C5" s="13" t="str">
+        <x:v>추가 요구 설계 동기화·구현 전</x:v>
+      </x:c>
+      <x:c r="D5" s="13" t="str">
+        <x:v>노트북 물리 계층, 혼합 Python 실행 페이지, NAS 원격 실행, PY/MD 로컬 투영, Markdown 표현 경계, 동적 자원 admission, 댓글/주석, 문서 스튜디오 Office 생성·첫 저장 위치·본문 reference UX를 관련 시트에 연결했다.</x:v>
+      </x:c>
+      <x:c r="E5" s="13" t="str">
+        <x:v>사용자 확인 9건과 릴레이 commits 12e28c3~f27bd79 대조. 실제 기능 구현·E2E는 아직 진행하지 않음.</x:v>
+      </x:c>
+      <x:c r="F5" s="13" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R081ec9f8de494055"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c8dd16b0fcc49df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7436,6 +8620,106 @@
       </x:c>
       <x:c r="F9" s="20" t="str">
         <x:v>IndexedDB/Yjs spike와 계정 로그아웃 cache purge gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="13" t="str">
+        <x:v>M1-F</x:v>
+      </x:c>
+      <x:c r="B10" s="13" t="str">
+        <x:v>노트북 물리 구조·페이지/일반 파일 계층</x:v>
+      </x:c>
+      <x:c r="C10" s="13" t="str">
+        <x:v>설계 확정·구현 전</x:v>
+      </x:c>
+      <x:c r="D10" s="13" t="str">
+        <x:v>NOTE MANAGER/노트북과 page marker, 하위 페이지·일반 파일 공존</x:v>
+      </x:c>
+      <x:c r="E10" s="13" t="str">
+        <x:v>미실시</x:v>
+      </x:c>
+      <x:c r="F10" s="13" t="str">
+        <x:v>현재 .note_studio 저장소와 파일 관리자 마이그레이션/호환 spike</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="13" t="str">
+        <x:v>M1-G</x:v>
+      </x:c>
+      <x:c r="B11" s="13" t="str">
+        <x:v>노트 본문 Office 생성·첫 저장·reference</x:v>
+      </x:c>
+      <x:c r="C11" s="13" t="str">
+        <x:v>설계 확정·구현 전</x:v>
+      </x:c>
+      <x:c r="D11" s="13" t="str">
+        <x:v>문서 스튜디오 재사용, invocation directory, stable document ID</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="str">
+        <x:v>미실시</x:v>
+      </x:c>
+      <x:c r="F11" s="13" t="str">
+        <x:v>공통 blank service 추출과 5개 형식 transaction/E2E</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="13" t="str">
+        <x:v>M1.5-A</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="str">
+        <x:v>페이지·블록·inline·코드 검토 댓글</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="str">
+        <x:v>설계 확정·구현 전</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="str">
+        <x:v>thread/anchor/mention/resolve 모델</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="str">
+        <x:v>미실시</x:v>
+      </x:c>
+      <x:c r="F12" s="13" t="str">
+        <x:v>Yjs/일반 revision 양쪽 anchor 이동 spike</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="13" t="str">
+        <x:v>M2-A</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>혼합 Python 실행 페이지·로컬 투영</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>설계 확정·구현 전</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="str">
+        <x:v>rich page + executable cells, PY+MD+manifest projection</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>미실시</x:v>
+      </x:c>
+      <x:c r="F13" s="13" t="str">
+        <x:v>nbformat/분리 파일 round-trip과 충돌 테스트</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="13" t="str">
+        <x:v>M2-B</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="str">
+        <x:v>NAS 원격 실행·동적 자원 scheduler</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="str">
+        <x:v>실장비 기준 확인·구현 전</x:v>
+      </x:c>
+      <x:c r="D14" s="13" t="str">
+        <x:v>cgroup v2, 전역/계정 active 1 초안, MASTER 고부하 capability</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>CPU/RAM/swap/disk/GPU 읽기 전용 확인</x:v>
+      </x:c>
+      <x:c r="F14" s="13" t="str">
+        <x:v>격리 worker·fair queue·부하/OOM/재감지 gate</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7647,7 +8931,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02a4050f64f7483d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d1b13a347e54b6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7930,7 +9214,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bfcaa8197a745bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc65f6620f3044e8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8326,7 +9610,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c3f4580832d4e87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb43ba7264eae4d2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8569,7 +9853,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra56b5799f0ea49f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63f98197dcc14041"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8744,7 +10028,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73e27692fb5b4828"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec22f17b39c84136"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8950,10 +10234,61 @@
         <x:v>다른 계정 링크면 자동 전환 금지, 사용자 선택. 앱 없으면 웹 fallback.</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="13" t="str">
+        <x:v>FLOW-PY-PROJECTION</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="str">
+        <x:v>NAS Drive에서 Python 실행 페이지 동기화</x:v>
+      </x:c>
+      <x:c r="C12" s="13" t="str">
+        <x:v>서버 page revision 확인 → .py/.md/assets/manifest 생성 또는 3-way 병합 → hash 기록</x:v>
+      </x:c>
+      <x:c r="D12" s="13" t="str">
+        <x:v>로컬 도구에서 순수 파일로 열고 수정 내용을 대응 block/cell에 역반영</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="str">
+        <x:v>서버·로컬 동시 수정은 덮어쓰지 않고 코드/문서별 충돌 비교와 복구본 제공</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="13" t="str">
+        <x:v>FLOW-PY-REMOTE</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="str">
+        <x:v>VS Code·터미널·노트에서 NAS 실행</x:v>
+      </x:c>
+      <x:c r="C13" s="13" t="str">
+        <x:v>사용자·workspace·capability 확인 → 자원 예약/admission → 격리 worker → 출력 stream → artifact publish</x:v>
+      </x:c>
+      <x:c r="D13" s="13" t="str">
+        <x:v>NAS 경로를 유지한 채 결과·오류·생성 파일을 PC에 표시</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>자원 부족은 실패가 아니라 대기. timeout/OOM은 worker만 종료하고 편집 내용 보존</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="13" t="str">
+        <x:v>FLOW-OFFICE-INLINE</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="str">
+        <x:v>노트 본문 caret 또는 노트북 폴더 우클릭</x:v>
+      </x:c>
+      <x:c r="C14" s="13" t="str">
+        <x:v>형식 선택 → invocation directory를 가진 draft → 작성 → 첫 저장 위치 선택 → 원자 publish → reference block 삽입 → 편집 창 전면 열기</x:v>
+      </x:c>
+      <x:c r="D14" s="13" t="str">
+        <x:v>기본 위치는 명령 발생 폴더이며 다른 NAS 위치를 골라도 원래 위치의 링크가 같은 문서를 연다.</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>원래 폴더 이동은 stable ID로 재해석. 삭제·권한 상실이면 위치를 다시 요구하고 임의 fallback 금지</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4d1e967b9b74a17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf4e88a2adb24ce1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>